<commit_message>
post-release: complete ten-target TLS matrix
</commit_message>
<xml_diff>
--- a/demo/certificates.xlsx
+++ b/demo/certificates.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet'!$A$1:$G$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet'!$A$1:$G$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,13 +415,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -467,68 +467,90 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Старый портал</t>
+          <t>Предупреждение</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>expired.lab.local</t>
+          <t>warning.lab.local</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>8443</v>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>warning@lab.local</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unreachable</t>
-        </is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>19</v>
+      </c>
+      <c r="G2" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Самоподписанный</t>
+          <t>Почта OWA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>selfsigned.lab.local</t>
+          <t>expiring.lab.local</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>8443</v>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>petrov@lab.local</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Unreachable</t>
-        </is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Почта OWA</t>
+          <t>Старый портал</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>expiring.lab.local</t>
+          <t>expired.lab.local</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>8443</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>petrov@lab.local</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Unreachable</t>
-        </is>
+          <t>Expired</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -552,19 +574,25 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Unreachable</t>
-        </is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>364</v>
+      </c>
+      <c r="G5" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ошибка имени</t>
+          <t>Информационный срок</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>mismatch.lab.local</t>
+          <t>information.lab.local</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -572,38 +600,164 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>sidorov@lab.local</t>
+          <t>info@lab.local</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Unreachable</t>
-        </is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>49</v>
+      </c>
+      <c r="G6" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Ошибка имени</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>mismatch.lab.local</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>8443</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>sidorov@lab.local</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>364</v>
+      </c>
+      <c r="G7" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Wildcard</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>app.wild.lab.local</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>8443</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>wildcard@lab.local</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>364</v>
+      </c>
+      <c r="G8" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Цепочка</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>chain.lab.local</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>8443</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ca@lab.local</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>364</v>
+      </c>
+      <c r="G9" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Самоподписанный</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>selfsigned.lab.local</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>8443</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>364</v>
+      </c>
+      <c r="G10" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Недоступный сервис</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>dead.lab.local</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C11" t="n">
         <v>65534</v>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
         <is>
           <t>Unreachable</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G7"/>
+  <autoFilter ref="A1:G11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh certificate reports with full metadata
Expanded the demo certificate exports to include detailed certificate metadata, risk analysis, and remediation recommendations. The CSV and HTML reports were updated to reflect the new inventory structure, and the XLSX snapshot was regenerated to match the revised certificate assessment data.
</commit_message>
<xml_diff>
--- a/demo/certificates.xlsx
+++ b/demo/certificates.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Сертификаты" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet'!$A$1:$G$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сертификаты'!$A$1:$V$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,13 +27,76 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00155724"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00856404"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00A84200"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000C5460"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00721C24"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00383D41"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+        <bgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE5D0"/>
+        <bgColor rgb="00FFE5D0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1ECF1"/>
+        <bgColor rgb="00D1ECF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+        <bgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2E3E5"/>
+        <bgColor rgb="00E2E3E5"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -48,8 +111,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,148 +485,481 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="43" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="45" customWidth="1" min="21" max="21"/>
+    <col width="45" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Сервис</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Хост</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Порт</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Владелец</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Критичность</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>SAN</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Issuer</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Thumbprint (SHA-1)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Действует с</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Действует до</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Дней осталось</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Дней до окончания</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Цепочка</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Имя совпадает</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Self-signed</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Ключ</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Подпись</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Risk Score</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Уровень риска</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Проблемы</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Рекомендации</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Предупреждение</t>
+          <t>HR-портал</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>warning.lab.local</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>8443</v>
+          <t>chain.lab.local</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>8443</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>warning@lab.local</t>
+          <t>hr@lab.local</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>19</v>
-      </c>
-      <c r="G2" t="n">
-        <v>75</v>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>chain.lab.local</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>chain.lab.local</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Radar Lab Rogue CA</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>4C6AC2BC9834EE5D94FA3B7E66CAC9D1B9CD6CD7</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>25.08.2026</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>24.09.2027</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>365</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>untrusted</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>RSA 2048</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: self-signed certificate in certificate chain (_ssl.c:1010)</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Почта OWA</t>
+          <t>VPN</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>expiring.lab.local</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>8443</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>petrov@lab.local</t>
-        </is>
-      </c>
+          <t>warning.lab.local</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>8443</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>warning.lab.local</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>warning.lab.local</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Radar Lab Intermediate CA</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>4FC0C98A3B270C852D71C53FA08BA5F7F1F0C465</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>24.09.2025</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>19.10.2026</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>untrusted</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>RSA 2048</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G3" t="n">
-        <v>100</v>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Сертификат истекает через 25 дн.; Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010); Не назначен владелец сервиса</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Запланируйте перевыпуск и замену сертификата до даты окончания. Назначьте ответственного.; Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.; Назначьте ответственного в инвентаре, чтобы уведомления доходили до исполнителя.</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Старый портал</t>
+          <t>Почта OWA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>expired.lab.local</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>8443</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>expiring.lab.local</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>8443</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>petrov@lab.local</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Expired</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>-2</v>
-      </c>
-      <c r="G4" t="n">
-        <v>100</v>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>expiring.lab.local</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>expiring.lab.local</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Radar Lab Intermediate CA</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>321906FC68D4B8B0E24EB2B5AC266E1B7438B5B0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>24.09.2025</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>untrusted</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>RSA 2048</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Сертификат истекает через 5 дн.; Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010)</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Запланируйте перевыпуск и замену сертификата до даты окончания. Назначьте ответственного.; Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Основной веб</t>
+          <t>Портал</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -564,8 +967,10 @@
           <t>valid.lab.local</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>8443</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>8443</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -574,51 +979,203 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>valid.lab.local</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>valid.lab.local</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Radar Lab Intermediate CA</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>D33CA1D62FF31B12B86332BA33911209F8954572</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>24.09.2025</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>12.04.2027</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>364</v>
-      </c>
-      <c r="G5" t="n">
-        <v>55</v>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>untrusted</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>RSA 2048</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010)</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Информационный срок</t>
+          <t>Legacy App</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>information.lab.local</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>8443</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>info@lab.local</t>
-        </is>
-      </c>
+          <t>weak.lab.local</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>8443</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Information</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>49</v>
-      </c>
-      <c r="G6" t="n">
-        <v>45</v>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>weak.lab.local</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>weak.lab.local</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>00869CCE4B70161B164CA928E53723F66A34E8A8</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>24.09.2026</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>24.09.2027</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>364</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>untrusted</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>RSA 1024</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>sha1</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: EE certificate key too weak (_ssl.c:1010); Слабый ключ: 1024 бит; Устаревший алгоритм подписи: sha1; Не назначен владелец сервиса</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.; Перевыпустите сертификат с ключом RSA не менее 2048 бит или ECDSA P-256.; Перевыпустите сертификат с подписью SHA-256 или выше.; Назначьте ответственного в инвентаре, чтобы уведомления доходили до исполнителя.</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ошибка имени</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -626,92 +1183,331 @@
           <t>mismatch.lab.local</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>8443</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>8443</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>sidorov@lab.local</t>
+          <t>api@lab.local</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>other.lab.local</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>other.lab.local</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Radar Lab Intermediate CA</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>D3F6D878B24D9A88CFE534600CBE78BD68C738C2</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>25.08.2026</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>24.09.2027</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>365</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>364</v>
-      </c>
-      <c r="G7" t="n">
-        <v>80</v>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>untrusted</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>RSA 2048</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010); Имя mismatch.lab.local не совпадает с CN/SAN сертификата: other.lab.local</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.; Перевыпустите сертификат с корректным именем в SAN или исправьте привязку сертификата на сервисе.</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wildcard</t>
+          <t>Wiki</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>app.wild.lab.local</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>8443</v>
+          <t>info.lab.local</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>8443</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>wildcard@lab.local</t>
+          <t>sidorov@lab.local</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>364</v>
-      </c>
-      <c r="G8" t="n">
-        <v>35</v>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>info.lab.local</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>info.lab.local</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Radar Lab Intermediate CA</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>6B049FA011FF40F68B0923289AC53130D647C317</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>24.09.2025</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>08.11.2026</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>untrusted</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>RSA 2048</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Сертификат истекает через 45 дн.; Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010)</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Запланируйте перевыпуск и замену сертификата до даты окончания. Назначьте ответственного.; Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Цепочка</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>chain.lab.local</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>8443</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>ca@lab.local</t>
-        </is>
-      </c>
+          <t>expired.lab.local</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>8443</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>364</v>
-      </c>
-      <c r="G9" t="n">
-        <v>35</v>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>expired.lab.local</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>expired.lab.local</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Radar Lab Intermediate CA</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>FB21A243B3549C444955C7A3401BAB2C531A78A1</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>20.08.2025</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>19.09.2026</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>Expired</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>untrusted</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>RSA 2048</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Срок действия сертификата истёк 5 дн. назад; Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010); Не назначен владелец сервиса</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Срочно перевыпустите сертификат и установите его на сервис. Проверьте, не нарушена ли работа клиентов.; Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.; Назначьте ответственного в инвентаре, чтобы уведомления доходили до исполнителя.</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Самоподписанный</t>
+          <t>Jenkins</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -719,26 +1515,111 @@
           <t>selfsigned.lab.local</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>8443</v>
-      </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>8443</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ops@lab.local</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>selfsigned.lab.local</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>selfsigned.lab.local</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>selfsigned.lab.local</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>F3DE868B60397C46CC76437FC151BAF1DE0E1264</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>25.08.2026</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>24.09.2027</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>365</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>364</v>
-      </c>
-      <c r="G10" t="n">
-        <v>50</v>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>self_signed</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>RSA 2048</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Сертификат самоподписанный, клиенты не могут проверить его подлинность</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Замените сертификат на выпущенный корпоративным или публичным центром сертификации.</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Недоступный сервис</t>
+          <t>Old Service</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -746,18 +1627,61 @@
           <t>dead.lab.local</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>65534</v>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>8499</t>
+        </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
           <t>Unreachable</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>untrusted</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Сервис недоступен: Таймаут соединения</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Проверьте доступность хоста и порта, правила межсетевого экрана и корректность DNS-имени.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G11"/>
+  <autoFilter ref="A1:V11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: finalize ui/ux v2, demo runbook, interactive presentation, and windows reliability
</commit_message>
<xml_diff>
--- a/demo/certificates.xlsx
+++ b/demo/certificates.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Сертификаты" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сертификаты'!$A$1:$V$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сертификаты'!$A$1:$Y$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +32,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00155724"/>
+      <color rgb="00721C24"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000C5460"/>
     </font>
     <font>
       <b val="1"/>
@@ -40,15 +44,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00A84200"/>
+      <color rgb="00155724"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000C5460"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00721C24"/>
+      <color rgb="00A84200"/>
     </font>
     <font>
       <b val="1"/>
@@ -64,8 +64,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
-        <bgColor rgb="00D4EDDA"/>
+        <fgColor rgb="00F8D7DA"/>
+        <bgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1ECF1"/>
+        <bgColor rgb="00D1ECF1"/>
       </patternFill>
     </fill>
     <fill>
@@ -76,20 +82,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE5D0"/>
-        <bgColor rgb="00FFE5D0"/>
+        <fgColor rgb="00D4EDDA"/>
+        <bgColor rgb="00D4EDDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D1ECF1"/>
-        <bgColor rgb="00D1ECF1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
-        <bgColor rgb="00F8D7DA"/>
+        <fgColor rgb="00FFE5D0"/>
+        <bgColor rgb="00FFE5D0"/>
       </patternFill>
     </fill>
     <fill>
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:Y11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -497,19 +497,22 @@
     <col width="23" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="43" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="45" customWidth="1" min="21" max="21"/>
-    <col width="45" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="45" customWidth="1" min="24" max="24"/>
+    <col width="45" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -560,65 +563,80 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Thumbprint (SHA-256)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Действует с</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Действует до</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Дней осталось</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Цепочка</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Имя совпадает</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Self-signed</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Ключ</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Подпись</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>TLS версия</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Ошибка</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Risk Score</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Уровень риска</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Проблемы</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Рекомендации</t>
         </is>
@@ -627,12 +645,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HR-портал</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>chain.lab.local</t>
+          <t>expired.lab.local</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -640,111 +658,118 @@
           <t>8443</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>hr@lab.local</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>chain.lab.local</t>
+          <t>expired.lab.local</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>chain.lab.local</t>
+          <t>expired.lab.local</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Radar Lab Rogue CA</t>
+          <t>Radar Lab Intermediate CA</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>4C6AC2BC9834EE5D94FA3B7E66CAC9D1B9CD6CD7</t>
+          <t>3F77EF749ADEA1C0739A1FDA5958B8D18956D3FA</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>25.08.2026</t>
+          <t>0525FE3B80727BF336B79F9F87B52FF6A735DA01A2EAE7F62FA3BED59385001E</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>24.09.2027</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>365</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>untrusted</t>
+          <t>19.09.2026</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Expired</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>trusted</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>RSA 2048</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: self-signed certificate in certificate chain (_ssl.c:1010)</t>
-        </is>
-      </c>
+          <t>TLSv1.3</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.</t>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Срок действия сертификата истёк 5 дн. назад; Не назначен владелец сервиса</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Срочно перевыпустите сертификат и установите его на сервис. Проверьте, не нарушена ли работа клиентов.; Назначьте ответственного в инвентаре, чтобы уведомления доходили до исполнителя.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VPN</t>
+          <t>Wiki</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>warning.lab.local</t>
+          <t>info.lab.local</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -752,20 +777,24 @@
           <t>8443</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>sidorov@lab.local</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>warning.lab.local</t>
+          <t>info.lab.local</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>warning.lab.local</t>
+          <t>info.lab.local</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -775,84 +804,95 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>4FC0C98A3B270C852D71C53FA08BA5F7F1F0C465</t>
+          <t>329758F89A3D2A650E175D0F645B8F8953A38195</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>3DA38BCAAC6303B664F7847B61DDADA6181B9062DE5D6C77045B35B75367CBD9</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>24.09.2025</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>19.10.2026</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>untrusted</t>
+          <t>08.11.2026</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Information</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>trusted</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>RSA 2048</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>95</t>
-        </is>
-      </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Сертификат истекает через 25 дн.; Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010); Не назначен владелец сервиса</t>
-        </is>
-      </c>
+          <t>TLSv1.3</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Запланируйте перевыпуск и замену сертификата до даты окончания. Назначьте ответственного.; Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.; Назначьте ответственного в инвентаре, чтобы уведомления доходили до исполнителя.</t>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Сертификат истекает через 45 дн.</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Запланируйте перевыпуск и замену сертификата до даты окончания. Назначьте ответственного.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Почта OWA</t>
+          <t>VPN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>expiring.lab.local</t>
+          <t>warning.lab.local</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -860,11 +900,7 @@
           <t>8443</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>petrov@lab.local</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>high</t>
@@ -872,12 +908,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>expiring.lab.local</t>
+          <t>warning.lab.local</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>expiring.lab.local</t>
+          <t>warning.lab.local</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -887,72 +923,83 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>321906FC68D4B8B0E24EB2B5AC266E1B7438B5B0</t>
+          <t>8DEEF85BF0C9D9C37F2D667FD1893E53F57580BE</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
+          <t>1FCAA6F519DD7725818088FD841CFE06CF0CE424643044C8D459420DE542461A</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>24.09.2025</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>29.09.2026</t>
-        </is>
-      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>untrusted</t>
+          <t>19.10.2026</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Warning</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>trusted</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>RSA 2048</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Сертификат истекает через 5 дн.; Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010)</t>
-        </is>
-      </c>
+          <t>TLSv1.3</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Запланируйте перевыпуск и замену сертификата до даты окончания. Назначьте ответственного.; Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.</t>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Сертификат истекает через 25 дн.; Не назначен владелец сервиса</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Запланируйте перевыпуск и замену сертификата до даты окончания. Назначьте ответственного.; Назначьте ответственного в инвентаре, чтобы уведомления доходили до исполнителя.</t>
         </is>
       </c>
     </row>
@@ -999,84 +1046,87 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>D33CA1D62FF31B12B86332BA33911209F8954572</t>
+          <t>AA34712445328FD53E97ACE7E7B8C2196C9DADB3</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
+          <t>1A1210CB61C40F6A00A1BDD04716B31CCF62E663A410A7BB975EF0FC149B49A5</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>24.09.2025</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>12.04.2027</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>untrusted</t>
-        </is>
-      </c>
       <c r="O5" t="inlineStr">
         <is>
+          <t>trusted</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>RSA 2048</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010)</t>
-        </is>
-      </c>
+          <t>TLSv1.3</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.</t>
-        </is>
-      </c>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Legacy App</t>
+          <t>Jenkins</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>weak.lab.local</t>
+          <t>selfsigned.lab.local</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1084,103 +1134,122 @@
           <t>8443</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ops@lab.local</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>weak.lab.local</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>selfsigned.lab.local</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>selfsigned.lab.local</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>weak.lab.local</t>
+          <t>selfsigned.lab.local</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>00869CCE4B70161B164CA928E53723F66A34E8A8</t>
+          <t>1ABAC377C46B5F270227308042BF477B9E3AD20A</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>24.09.2026</t>
+          <t>3201275A9D62802569E9FCA20F1B91D5E9F31630265EDAE06CCCE4BAA6A8E995</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>25.08.2026</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
           <t>24.09.2027</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>364</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>365</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>untrusted</t>
-        </is>
-      </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>self_signed</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>RSA 1024</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>sha1</t>
+          <t>RSA 2048</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>sha256</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: EE certificate key too weak (_ssl.c:1010); Слабый ключ: 1024 бит; Устаревший алгоритм подписи: sha1; Не назначен владелец сервиса</t>
-        </is>
-      </c>
+          <t>TLSv1.3</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.; Перевыпустите сертификат с ключом RSA не менее 2048 бит или ECDSA P-256.; Перевыпустите сертификат с подписью SHA-256 или выше.; Назначьте ответственного в инвентаре, чтобы уведомления доходили до исполнителя.</t>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Сертификат самоподписанный, клиенты не могут проверить его подлинность</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Замените сертификат на выпущенный корпоративным или публичным центром сертификации.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>HR-портал</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>mismatch.lab.local</t>
+          <t>chain.lab.local</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1190,109 +1259,120 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>api@lab.local</t>
+          <t>hr@lab.local</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>other.lab.local</t>
+          <t>chain.lab.local</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>other.lab.local</t>
+          <t>chain.lab.local</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Radar Lab Intermediate CA</t>
+          <t>Radar Lab Rogue CA</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>D3F6D878B24D9A88CFE534600CBE78BD68C738C2</t>
+          <t>896EDB0325F6CF3B2D1A5F17392407683E763C25</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
+          <t>A167F3DB75A1CE2FFDB7C16A764640AE1243CFF72CC1AB1C1777020D14D580F4</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
           <t>25.08.2026</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>24.09.2027</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>365</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>untrusted</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>RSA 2048</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010); Имя mismatch.lab.local не совпадает с CN/SAN сертификата: other.lab.local</t>
-        </is>
-      </c>
+          <t>TLSv1.3</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.; Перевыпустите сертификат с корректным именем в SAN или исправьте привязку сертификата на сервисе.</t>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: self-signed certificate in certificate chain (_ssl.c:1010)</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wiki</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>info.lab.local</t>
+          <t>mismatch.lab.local</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1302,22 +1382,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>sidorov@lab.local</t>
+          <t>api@lab.local</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>info.lab.local</t>
+          <t>other.lab.local</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>info.lab.local</t>
+          <t>other.lab.local</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1327,37 +1407,37 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>6B049FA011FF40F68B0923289AC53130D647C317</t>
+          <t>6B5D77F9604A8BE0CEB864B8719B8AF1FB06FFA3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>24.09.2025</t>
+          <t>565707BB97AB4F3CD3F8D4714B4903BFEEF6773716359B5C32495DC05593A02F</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>08.11.2026</t>
+          <t>25.08.2026</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>Information</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>untrusted</t>
+          <t>24.09.2027</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>365</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>trusted</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1367,44 +1447,55 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
           <t>RSA 2048</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
       <c r="T8" t="inlineStr">
         <is>
+          <t>TLSv1.3</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Сертификат истекает через 45 дн.; Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010)</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>Запланируйте перевыпуск и замену сертификата до даты окончания. Назначьте ответственного.; Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.</t>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Имя mismatch.lab.local не совпадает с CN/SAN сертификата: other.lab.local</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Перевыпустите сертификат с корректным именем в SAN или исправьте привязку сертификата на сервисе.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Почта OWA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>expired.lab.local</t>
+          <t>expiring.lab.local</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1412,7 +1503,11 @@
           <t>8443</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>petrov@lab.local</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>high</t>
@@ -1420,12 +1515,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>expired.lab.local</t>
+          <t>expiring.lab.local</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>expired.lab.local</t>
+          <t>expiring.lab.local</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1435,84 +1530,95 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>FB21A243B3549C444955C7A3401BAB2C531A78A1</t>
+          <t>CEBBE7317B34F062434ED05718EC12853F066A3E</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>40664BA229989E777C18A5BBA63DB1C00193F5921A1C02AD9620291D17BAFE37</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>19.09.2026</t>
+          <t>24.09.2025</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>-5</t>
-        </is>
-      </c>
-      <c r="M9" s="6" t="inlineStr">
-        <is>
-          <t>Expired</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>untrusted</t>
+          <t>29.09.2026</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
+          <t>trusted</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>RSA 2048</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
       <c r="T9" t="inlineStr">
         <is>
+          <t>TLSv1.3</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Срок действия сертификата истёк 5 дн. назад; Ошибка цепочки доверия: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: certificate signature failure (_ssl.c:1010); Не назначен владелец сервиса</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Срочно перевыпустите сертификат и установите его на сервис. Проверьте, не нарушена ли работа клиентов.; Установите на сервере полную цепочку (промежуточные сертификаты) или используйте сертификат доверенного центра сертификации.; Назначьте ответственного в инвентаре, чтобы уведомления доходили до исполнителя.</t>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Сертификат истекает через 5 дн.</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Запланируйте перевыпуск и замену сертификата до даты окончания. Назначьте ответственного.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jenkins</t>
+          <t>Legacy App</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>selfsigned.lab.local</t>
+          <t>weak.lab.local</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1520,99 +1626,106 @@
           <t>8443</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>ops@lab.local</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>selfsigned.lab.local</t>
+          <t>weak.lab.local</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>selfsigned.lab.local</t>
+          <t>weak.lab.local</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>selfsigned.lab.local</t>
+          <t>weak.lab.local</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>F3DE868B60397C46CC76437FC151BAF1DE0E1264</t>
+          <t>8F9869C708F49DA0500DAAF602D1B14F4C3AFE0A</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
+          <t>F7EF191D3C86AD16EF7E6524AFCE06E8D10F3CBBD888ECE733BA5C9FDBBA025A</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
           <t>25.08.2026</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>24.09.2027</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>365</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>self_signed</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>RSA 2048</t>
-        </is>
-      </c>
       <c r="R10" t="inlineStr">
         <is>
+          <t>RSA 1024</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
       <c r="T10" t="inlineStr">
         <is>
+          <t>TLSv1.3</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Сертификат самоподписанный, клиенты не могут проверить его подлинность</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>Замените сертификат на выпущенный корпоративным или публичным центром сертификации.</t>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Сертификат самоподписанный, клиенты не могут проверить его подлинность; Слабый ключ: 1024 бит; Не назначен владелец сервиса</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Замените сертификат на выпущенный корпоративным или публичным центром сертификации.; Перевыпустите сертификат с ключом RSA не менее 2048 бит или ECDSA P-256.; Назначьте ответственного в инвентаре, чтобы уведомления доходили до исполнителя.</t>
         </is>
       </c>
     </row>
@@ -1645,43 +1758,50 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
-      <c r="M11" s="7" t="inlineStr">
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" s="7" t="inlineStr">
         <is>
           <t>Unreachable</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>untrusted</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr">
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr">
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Таймаут соединения</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>Сервис недоступен: Таймаут соединения</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="Y11" t="inlineStr">
         <is>
           <t>Проверьте доступность хоста и порта, правила межсетевого экрана и корректность DNS-имени.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V11"/>
+  <autoFilter ref="A1:Y11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>